<commit_message>
Tapeout budget: 5% margin for a rise of the exchange rate
</commit_message>
<xml_diff>
--- a/docs/anggaran_tapeout.xlsx
+++ b/docs/anggaran_tapeout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\stereo-depth-cam\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{308676DB-8167-4A1A-99CA-0A058078E56E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D03898-1DB1-4219-A607-46602B3E2B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="133">
   <si>
     <t>Anggaran tapeout Tiny Tapeout: asumsi dan sumber</t>
   </si>
@@ -154,6 +154,18 @@
     <t>DHL: aturan de minimis 2026 (ambang USD 3)</t>
   </si>
   <si>
+    <t>Margin kenaikan kurs</t>
+  </si>
+  <si>
+    <t>Cadangan bila rupiah melemah sebelum pembayaran (devkit dibayar sekarang, pajak impor dibayar saat chip tiba, sekitar Juni 2027)</t>
+  </si>
+  <si>
+    <t>Kurs yang dipakai menghitung (kurs x (1 + margin))</t>
+  </si>
+  <si>
+    <t>Semua konversi euro ke rupiah memakai kurs ini</t>
+  </si>
+  <si>
     <t>Papan interface ke EBAZ4205 (beli lokal / JLCPCB)</t>
   </si>
   <si>
@@ -244,6 +256,9 @@
     <t>TOTAL tanpa NPWP</t>
   </si>
   <si>
+    <t xml:space="preserve">  di dalamnya: cadangan margin kurs</t>
+  </si>
+  <si>
     <t>Biaya desain (8 petak) dibayar sekali; chip kedua berarti devkit kedua. Di chip Tiny Tapeout hanya satu proyek aktif pada satu waktu, jadi rantai 2 irisan butuh 2 chip fisik.</t>
   </si>
   <si>
@@ -313,7 +328,10 @@
     <t>TOTAL tanpa NPWP (PPh 20%)</t>
   </si>
   <si>
-    <t>TOTAL dengan NPWP, dalam euro (kurs asumsi)</t>
+    <t>TOTAL dengan NPWP, dalam euro (kurs dengan margin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  di dalamnya: cadangan dari margin kenaikan kurs</t>
   </si>
   <si>
     <t>Catatan: pin EBAZ4205 untuk hub (17 + N) belum tersedia dengan susunan sekarang; cek header J3/J5 sebelum membeli. Ketersediaan 4x2 dan harga SKY26d perlu dikonfirmasi di kalkulator saat memesan.</t>
@@ -548,7 +566,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -564,6 +582,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="167" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -891,7 +911,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
@@ -1103,141 +1123,170 @@
         <v>38</v>
       </c>
     </row>
+    <row r="16" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" s="10"/>
+    </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B18" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="B17" s="12">
+        <f>B9*(1+B16)</f>
+        <v>21525</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="E17" s="8"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="E20" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" s="12">
+    <row r="21" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" s="14">
         <v>100000</v>
       </c>
-      <c r="C19" s="13">
+      <c r="C21" s="15">
         <v>1</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" s="12">
-        <v>275000</v>
-      </c>
-      <c r="C20" s="13">
-        <v>1</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
+      <c r="D21" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B21" s="12">
-        <v>50000</v>
-      </c>
-      <c r="C21" s="13">
-        <v>1</v>
-      </c>
-      <c r="D21" s="4" t="s">
+      <c r="E21" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E21" s="10"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="12">
-        <v>10000</v>
-      </c>
-      <c r="C22" s="13">
+      <c r="B22" s="14">
+        <v>275000</v>
+      </c>
+      <c r="C22" s="15">
         <v>1</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E22" s="8" t="s">
-        <v>52</v>
+      <c r="E22" s="6" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="14">
+        <v>50000</v>
+      </c>
+      <c r="C23" s="15">
+        <v>1</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="12">
-        <v>25000</v>
-      </c>
-      <c r="C23" s="13">
-        <v>1</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>49</v>
-      </c>
       <c r="E23" s="10"/>
     </row>
-    <row r="24" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="12">
-        <v>200000</v>
-      </c>
-      <c r="C24" s="13">
-        <v>0</v>
+      <c r="B24" s="14">
+        <v>10000</v>
+      </c>
+      <c r="C24" s="15">
+        <v>1</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>55</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B25" s="14">
+        <v>25000</v>
+      </c>
+      <c r="C25" s="15">
+        <v>1</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E25" s="10"/>
+    </row>
+    <row r="26" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="14">
+        <v>200000</v>
+      </c>
+      <c r="C26" s="15">
+        <v>0</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E26" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B25" s="14">
-        <f>SUMPRODUCT(B19:B24,C19:C24)</f>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27" s="16">
+        <f>SUMPRODUCT(B21:B26,C21:C26)</f>
         <v>460000</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="B26" s="14">
-        <f>SUM(B19:B24)</f>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" s="16">
+        <f>SUM(B21:B26)</f>
         <v>660000</v>
       </c>
     </row>
@@ -1252,8 +1301,8 @@
     <hyperlink ref="E12" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
     <hyperlink ref="E13" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
     <hyperlink ref="E15" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="E19" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="E20" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="E21" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="E22" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1261,7 +1310,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
@@ -1270,142 +1319,159 @@
   <sheetData>
     <row r="1" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B4" s="15">
+        <v>67</v>
+      </c>
+      <c r="B4" s="17">
         <f>'1 IC'!D8</f>
-        <v>17937500</v>
-      </c>
-      <c r="C4" s="15">
+        <v>18834375</v>
+      </c>
+      <c r="C4" s="17">
         <f>'2 IC'!D8</f>
-        <v>24395000</v>
-      </c>
-      <c r="D4" s="16">
-        <f t="shared" ref="D4:D9" si="0">C4-B4</f>
-        <v>6457500</v>
+        <v>25614750</v>
+      </c>
+      <c r="D4" s="18">
+        <f t="shared" ref="D4:D10" si="0">C4-B4</f>
+        <v>6780375</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B5" s="15">
+        <v>68</v>
+      </c>
+      <c r="B5" s="17">
         <f>SUM('1 IC'!D10:D12)</f>
-        <v>1942093.125</v>
-      </c>
-      <c r="C5" s="15">
+        <v>2039197.78125</v>
+      </c>
+      <c r="C5" s="17">
         <f>SUM('2 IC'!D10:D12)</f>
-        <v>3884186.25</v>
-      </c>
-      <c r="D5" s="16">
+        <v>4078395.5625</v>
+      </c>
+      <c r="D5" s="18">
         <f t="shared" si="0"/>
-        <v>1942093.125</v>
+        <v>2039197.78125</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="B6" s="15">
+        <v>69</v>
+      </c>
+      <c r="B6" s="17">
         <f>'1 IC'!D13</f>
-        <v>538125</v>
-      </c>
-      <c r="C6" s="15">
+        <v>565031.25</v>
+      </c>
+      <c r="C6" s="17">
         <f>'2 IC'!D13</f>
-        <v>731850</v>
-      </c>
-      <c r="D6" s="16">
+        <v>768442.5</v>
+      </c>
+      <c r="D6" s="18">
         <f t="shared" si="0"/>
-        <v>193725</v>
+        <v>203411.25</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="B7" s="15">
+        <v>70</v>
+      </c>
+      <c r="B7" s="17">
         <f>'1 IC'!D14</f>
         <v>460000</v>
       </c>
-      <c r="C7" s="15">
+      <c r="C7" s="17">
         <f>'2 IC'!D14</f>
         <v>660000</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="18">
         <f t="shared" si="0"/>
         <v>200000</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="B8" s="18">
+      <c r="A8" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="20">
         <f>'1 IC'!D16</f>
-        <v>20877718.125</v>
-      </c>
-      <c r="C8" s="18">
+        <v>21898604.03125</v>
+      </c>
+      <c r="C8" s="20">
         <f>'2 IC'!D16</f>
-        <v>29671036.25</v>
-      </c>
-      <c r="D8" s="19">
+        <v>31121588.0625</v>
+      </c>
+      <c r="D8" s="21">
         <f t="shared" si="0"/>
-        <v>8793318.125</v>
+        <v>9222984.03125</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="18">
+      <c r="A9" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B9" s="20">
         <f>'1 IC'!D17</f>
-        <v>21571899.375</v>
-      </c>
-      <c r="C9" s="18">
+        <v>22627494.34375</v>
+      </c>
+      <c r="C9" s="20">
         <f>'2 IC'!D17</f>
-        <v>31059398.75</v>
-      </c>
-      <c r="D9" s="19">
+        <v>32579368.6875</v>
+      </c>
+      <c r="D9" s="21">
         <f t="shared" si="0"/>
-        <v>9487499.375</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="B11" s="29"/>
-      <c r="C11" s="29"/>
-      <c r="D11" s="29"/>
+        <v>9951874.34375</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="17">
+        <f>'1 IC'!D19</f>
+        <v>1020885.90625</v>
+      </c>
+      <c r="C10" s="17">
+        <f>'2 IC'!D19</f>
+        <v>1450551.8125</v>
+      </c>
+      <c r="D10" s="18">
+        <f t="shared" si="0"/>
+        <v>429665.90625</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="29"/>
-      <c r="B12" s="29"/>
-      <c r="C12" s="29"/>
-      <c r="D12" s="29"/>
+      <c r="A12" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="31"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="31"/>
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A11:D12"/>
+    <mergeCell ref="A12:D13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1413,7 +1479,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -1425,128 +1491,128 @@
   <sheetData>
     <row r="1" spans="1:5" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B5" s="20">
+        <v>80</v>
+      </c>
+      <c r="B5" s="22">
         <f>Asumsi!$B$6</f>
         <v>8</v>
       </c>
-      <c r="C5" s="21">
+      <c r="C5" s="23">
         <f>B5*Asumsi!$B$5</f>
         <v>560</v>
       </c>
-      <c r="D5" s="16">
-        <f>C5*Asumsi!$B$9</f>
-        <v>11480000</v>
+      <c r="D5" s="18">
+        <f>C5*Asumsi!$B$17</f>
+        <v>12054000</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B6" s="13">
+        <v>82</v>
+      </c>
+      <c r="B6" s="15">
         <v>1</v>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="23">
         <f>B6*Asumsi!$B$7</f>
         <v>300</v>
       </c>
-      <c r="D6" s="16">
-        <f>C6*Asumsi!$B$9</f>
-        <v>6150000</v>
+      <c r="D6" s="18">
+        <f>C6*Asumsi!$B$17</f>
+        <v>6457500</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B7" s="13">
+        <v>84</v>
+      </c>
+      <c r="B7" s="15">
         <v>1</v>
       </c>
-      <c r="C7" s="21">
+      <c r="C7" s="23">
         <f>B7*Asumsi!$B$8</f>
         <v>15</v>
       </c>
-      <c r="D7" s="16">
-        <f>C7*Asumsi!$B$9</f>
-        <v>307500</v>
+      <c r="D7" s="18">
+        <f>C7*Asumsi!$B$17</f>
+        <v>322875</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="22" t="s">
-        <v>81</v>
+      <c r="A8" s="24" t="s">
+        <v>86</v>
       </c>
       <c r="B8" s="8"/>
-      <c r="C8" s="23">
+      <c r="C8" s="25">
         <f>SUM(C5:C7)</f>
         <v>875</v>
       </c>
-      <c r="D8" s="24">
+      <c r="D8" s="26">
         <f>SUM(D5:D7)</f>
-        <v>17937500</v>
+        <v>18834375</v>
       </c>
       <c r="E8" s="4"/>
     </row>
     <row r="9" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
-      <c r="D9" s="16">
+      <c r="D9" s="18">
         <f>D6+D7</f>
-        <v>6457500</v>
+        <v>6780375</v>
       </c>
       <c r="E9" s="4"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
-      <c r="D10" s="16">
+      <c r="D10" s="18">
         <f>D9*Asumsi!$B$10</f>
-        <v>484312.5</v>
+        <v>508528.125</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -1555,26 +1621,26 @@
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
-      <c r="D11" s="16">
+      <c r="D11" s="18">
         <f>(D9+D10)*Asumsi!$B$11</f>
-        <v>763599.375</v>
+        <v>801779.34375</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
-      <c r="D12" s="16">
+      <c r="D12" s="18">
         <f>(D9+D10)*Asumsi!$B$12</f>
-        <v>694181.25</v>
+        <v>728890.3125</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -1583,26 +1649,26 @@
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
-      <c r="D13" s="16">
+      <c r="D13" s="18">
         <f>D8*Asumsi!$B$14</f>
-        <v>538125</v>
+        <v>565031.25</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
-      <c r="D14" s="16">
-        <f>Asumsi!$B$25</f>
+      <c r="D14" s="18">
+        <f>Asumsi!$B$27</f>
         <v>460000</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -1613,60 +1679,72 @@
       <c r="E15" s="4"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="25" t="s">
-        <v>90</v>
+      <c r="A16" s="27" t="s">
+        <v>95</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
-      <c r="D16" s="26">
+      <c r="D16" s="28">
         <f>D8+SUM(D10:D14)</f>
-        <v>20877718.125</v>
+        <v>21898604.03125</v>
       </c>
       <c r="E16" s="4"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="25" t="s">
-        <v>91</v>
+      <c r="A17" s="27" t="s">
+        <v>96</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
-      <c r="D17" s="26">
+      <c r="D17" s="28">
         <f>D16-D12+(D9+D10)*Asumsi!$B$13</f>
-        <v>21571899.375</v>
+        <v>22627494.34375</v>
       </c>
       <c r="E17" s="4"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="25" t="s">
-        <v>92</v>
+      <c r="A18" s="27" t="s">
+        <v>97</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
-      <c r="D18" s="27">
-        <f>D16/Asumsi!$B$9</f>
-        <v>1018.4252743902439</v>
+      <c r="D18" s="29">
+        <f>D16/Asumsi!$B$17</f>
+        <v>1017.3567494192799</v>
       </c>
       <c r="E18" s="4"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="B20" s="29"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="18">
+        <f>(D16-D14)*Asumsi!$B$16/(1+Asumsi!$B$16)</f>
+        <v>1020885.90625</v>
+      </c>
+      <c r="E19" s="4"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="29"/>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29"/>
+      <c r="A21" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="B21" s="31"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="31"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A20:E21"/>
+    <mergeCell ref="A21:E22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1674,7 +1752,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -1686,128 +1764,128 @@
   <sheetData>
     <row r="1" spans="1:5" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B5" s="20">
+        <v>80</v>
+      </c>
+      <c r="B5" s="22">
         <f>Asumsi!$B$6</f>
         <v>8</v>
       </c>
-      <c r="C5" s="21">
+      <c r="C5" s="23">
         <f>B5*Asumsi!$B$5</f>
         <v>560</v>
       </c>
-      <c r="D5" s="16">
-        <f>C5*Asumsi!$B$9</f>
-        <v>11480000</v>
+      <c r="D5" s="18">
+        <f>C5*Asumsi!$B$17</f>
+        <v>12054000</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B6" s="13">
+        <v>82</v>
+      </c>
+      <c r="B6" s="15">
         <v>2</v>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="23">
         <f>B6*Asumsi!$B$7</f>
         <v>600</v>
       </c>
-      <c r="D6" s="16">
-        <f>C6*Asumsi!$B$9</f>
-        <v>12300000</v>
+      <c r="D6" s="18">
+        <f>C6*Asumsi!$B$17</f>
+        <v>12915000</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B7" s="13">
+        <v>84</v>
+      </c>
+      <c r="B7" s="15">
         <v>2</v>
       </c>
-      <c r="C7" s="21">
+      <c r="C7" s="23">
         <f>B7*Asumsi!$B$8</f>
         <v>30</v>
       </c>
-      <c r="D7" s="16">
-        <f>C7*Asumsi!$B$9</f>
-        <v>615000</v>
+      <c r="D7" s="18">
+        <f>C7*Asumsi!$B$17</f>
+        <v>645750</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="22" t="s">
-        <v>81</v>
+      <c r="A8" s="24" t="s">
+        <v>86</v>
       </c>
       <c r="B8" s="8"/>
-      <c r="C8" s="23">
+      <c r="C8" s="25">
         <f>SUM(C5:C7)</f>
         <v>1190</v>
       </c>
-      <c r="D8" s="24">
+      <c r="D8" s="26">
         <f>SUM(D5:D7)</f>
-        <v>24395000</v>
+        <v>25614750</v>
       </c>
       <c r="E8" s="4"/>
     </row>
     <row r="9" spans="1:5" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
-      <c r="D9" s="16">
+      <c r="D9" s="18">
         <f>D6+D7</f>
-        <v>12915000</v>
+        <v>13560750</v>
       </c>
       <c r="E9" s="4"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
-      <c r="D10" s="16">
+      <c r="D10" s="18">
         <f>D9*Asumsi!$B$10</f>
-        <v>968625</v>
+        <v>1017056.25</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -1816,26 +1894,26 @@
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
-      <c r="D11" s="16">
+      <c r="D11" s="18">
         <f>(D9+D10)*Asumsi!$B$11</f>
-        <v>1527198.75</v>
+        <v>1603558.6875</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
-      <c r="D12" s="16">
+      <c r="D12" s="18">
         <f>(D9+D10)*Asumsi!$B$12</f>
-        <v>1388362.5</v>
+        <v>1457780.625</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -1844,26 +1922,26 @@
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
-      <c r="D13" s="16">
+      <c r="D13" s="18">
         <f>D8*Asumsi!$B$14</f>
-        <v>731850</v>
+        <v>768442.5</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
-      <c r="D14" s="16">
-        <f>Asumsi!$B$26</f>
+      <c r="D14" s="18">
+        <f>Asumsi!$B$28</f>
         <v>660000</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -1874,60 +1952,72 @@
       <c r="E15" s="4"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="25" t="s">
-        <v>90</v>
+      <c r="A16" s="27" t="s">
+        <v>95</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
-      <c r="D16" s="26">
+      <c r="D16" s="28">
         <f>D8+SUM(D10:D14)</f>
-        <v>29671036.25</v>
+        <v>31121588.0625</v>
       </c>
       <c r="E16" s="4"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="25" t="s">
-        <v>91</v>
+      <c r="A17" s="27" t="s">
+        <v>96</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
-      <c r="D17" s="26">
+      <c r="D17" s="28">
         <f>D16-D12+(D9+D10)*Asumsi!$B$13</f>
-        <v>31059398.75</v>
+        <v>32579368.6875</v>
       </c>
       <c r="E17" s="4"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="25" t="s">
-        <v>92</v>
+      <c r="A18" s="27" t="s">
+        <v>97</v>
       </c>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
-      <c r="D18" s="27">
-        <f>D16/Asumsi!$B$9</f>
-        <v>1447.3676219512195</v>
+      <c r="D18" s="29">
+        <f>D16/Asumsi!$B$17</f>
+        <v>1445.8345209059235</v>
       </c>
       <c r="E18" s="4"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="B20" s="29"/>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
-      <c r="E20" s="29"/>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="18">
+        <f>(D16-D14)*Asumsi!$B$16/(1+Asumsi!$B$16)</f>
+        <v>1450551.8125</v>
+      </c>
+      <c r="E19" s="4"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="29"/>
-      <c r="B21" s="29"/>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29"/>
+      <c r="A21" s="30" t="s">
+        <v>99</v>
+      </c>
+      <c r="B21" s="31"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="31"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A20:E21"/>
+    <mergeCell ref="A21:E22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1945,7 +2035,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -1953,10 +2043,10 @@
         <v>6</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -1964,43 +2054,43 @@
         <v>10</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -2008,21 +2098,21 @@
         <v>25</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -2030,10 +2120,10 @@
         <v>38</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -2041,10 +2131,10 @@
         <v>28</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -2052,32 +2142,32 @@
         <v>22</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -2085,15 +2175,15 @@
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>